<commit_message>
refactor: Remove diacritics, consolidate VBA into single module
- Remove all Romanian diacritics (ă,î,ș,ț,â) to avoid display issues
- Consolidate 3 VBA files into single ModNecesar.bas
- Setup simplified to: import 1 file + run 1 macro
- Regenerate Excel and templates without diacritics

https://claude.ai/code/session_01WLPgVpN32fAC7hpn167gUT
</commit_message>
<xml_diff>
--- a/NecesarAprovizionare.xlsx
+++ b/NecesarAprovizionare.xlsx
@@ -578,13 +578,13 @@
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>▶  IMPORT STOC DEPOZIT</t>
+          <t>IMPORT STOC DEPOZIT</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Importă fișierul cu stocul din depozit.
-Format: Cod Produs | Stoc</t>
+          <t>Importa fisierul cu stocul din depozit.
+Format: CodProdus | Stoc</t>
         </is>
       </c>
     </row>
@@ -592,13 +592,13 @@
     <row r="10">
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>▶  IMPORT VÂNZĂRI MAGAZIN</t>
+          <t>IMPORT VANZARI MAGAZIN</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Importă fișierul cu vânzările magazinului.
-Format: Cod Produs | Cantitate Vânzare</t>
+          <t>Importa fisierul cu vanzarile magazinului.
+Format: CodProdus | Cantitate</t>
         </is>
       </c>
     </row>
@@ -606,20 +606,20 @@
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>ACȚIUNI RAPIDE</t>
+          <t>ACTIUNI RAPIDE</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>✕  ȘTERGE TOATE DATELE</t>
+          <t>STERGE TOATE DATELE</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Șterge toate datele importate.
-Folosește pentru a reîncepe procesul.</t>
+          <t>Sterge toate datele importate.
+Foloseste pentru a reincepe procesul.</t>
         </is>
       </c>
     </row>
@@ -639,19 +639,19 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>⊘ Neîncărcat</t>
+          <t>Neincarcat</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Vânzări Magazin:</t>
+          <t>Vanzari Magazin:</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>⊘ Neîncărcat</t>
+          <t>Neincarcat</t>
         </is>
       </c>
     </row>
@@ -670,42 +670,42 @@
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>INSTRUCȚIUNI</t>
+          <t>INSTRUCTIUNI</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>1. Pregătiți fișierele de import conform șabloanelor din folderul 'Sabloane'.</t>
+          <t>1. Pregatiti fisierele de import conform sabloanelor din folderul 'sabloane'.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>2. Fișierul de stoc trebuie să aibă headerul: CodProdus | Stoc</t>
+          <t>2. Fisierul de stoc trebuie sa aiba headerul: CodProdus | Stoc</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>3. Fișierul de vânzări trebuie să aibă headerul: CodProdus | Cantitate</t>
+          <t>3. Fisierul de vanzari trebuie sa aiba headerul: CodProdus | Cantitate</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>4. Apăsați butonul corespunzător sau folosiți meniul "Necesar" din bara de sus.</t>
+          <t>4. Apasati butonul corespunzator pentru a importa datele.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>5. Selectați fișierul .xlsx și așteptați confirmarea importului.</t>
+          <t>5. Selectati fisierul .xlsx si asteptati confirmarea importului.</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>Cantitate Vânzare</t>
+          <t>Cantitate Vanzare</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="C1" s="12" t="inlineStr">
         <is>
-          <t>Observații</t>
+          <t>Observatii</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>Unitate Măsură</t>
+          <t>Unitate Masura</t>
         </is>
       </c>
       <c r="C1" s="12" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>Operațiune</t>
+          <t>Operatiune</t>
         </is>
       </c>
       <c r="C1" s="12" t="inlineStr">

</xml_diff>

<commit_message>
feat: Add GenerareNecesar, compatibility, rounding rules, 2000-product templates
Major update:
- Silent VBA operations (no focus changes, minimal messages)
- Single confirmation only for delete, no confirmation for imports
- GenerareNecesar: calculates supply needs from sales data
  - Applies product compatibility replacements (code substitution)
  - Applies 4 rounding categories (multiples of 10/2/5, min thresholds)
  - Aggregates quantities when multiple codes map to same compatible code
  - Shows observations: compatibility changes and rounding applied
- ReguliRotunjire: two-section layout (categories + product assignments)
- Necesar output sheet with Cod/Vanzare/Necesar/Observatii columns
- Templates updated to 2000 products with integer quantities
- All text without diacritics

https://claude.ai/code/session_01WLPgVpN32fAC7hpn167gUT
</commit_message>
<xml_diff>
--- a/NecesarAprovizionare.xlsx
+++ b/NecesarAprovizionare.xlsx
@@ -12,13 +12,14 @@
     <sheet name="VanzariMagazin" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Compatibilitati" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="ReguliRotunjire" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Log" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Necesar" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Log" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'StocDepozit'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'VanzariMagazin'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Compatibilitati'!$A$1:$C$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ReguliRotunjire'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Compatibilitati'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Necesar'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,8 +95,17 @@
       <i val="1"/>
       <color rgb="00999999"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -116,6 +126,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="006A1B9A"/>
+        <bgColor rgb="006A1B9A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00C62828"/>
         <bgColor rgb="00C62828"/>
       </patternFill>
@@ -124,6 +140,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="002F5496"/>
         <bgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F57C00"/>
+        <bgColor rgb="00F57C00"/>
       </patternFill>
     </fill>
   </fills>
@@ -145,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -166,19 +188,29 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -545,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C30"/>
+  <dimension ref="B2:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -583,8 +615,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Importa fisierul cu stocul din depozit.
-Format: CodProdus | Stoc</t>
+          <t>Importa stocul din depozit. Format: CodProdus | Stoc</t>
         </is>
       </c>
     </row>
@@ -597,8 +628,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Importa fisierul cu vanzarile magazinului.
-Format: CodProdus | Cantitate</t>
+          <t>Importa vanzarile magazinului. Format: CodProdus | Cantitate</t>
         </is>
       </c>
     </row>
@@ -606,128 +636,154 @@
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>ACTIUNI RAPIDE</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="7" t="inlineStr">
+          <t>PASUL 2: GENERARE NECESAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>GENERARE NECESAR</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Calculeaza necesarul cu compatibilitati si rotunjiri.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>ACTIUNI</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>STERGE TOATE DATELE</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Sterge toate datele importate.
-Foloseste pentru a reincepe procesul.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
-    <row r="18">
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>STATUS IMPORT</t>
-        </is>
-      </c>
-    </row>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Sterge datele importate si necesarul generat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
     <row r="20">
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Stoc Depozit:</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>Neincarcat</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Vanzari Magazin:</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Neincarcat</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Ultima actualizare:</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Necesar:</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Negenerat</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>INSTRUCTIUNI</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>1. Pregatiti fisierele de import conform sabloanelor din folderul 'sabloane'.</t>
-        </is>
-      </c>
-    </row>
     <row r="27">
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>2. Fisierul de stoc trebuie sa aiba headerul: CodProdus | Stoc</t>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>1. Importati stocul si vanzarile folosind butoanele de mai sus.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>3. Fisierul de vanzari trebuie sa aiba headerul: CodProdus | Cantitate</t>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>2. Fisierele trebuie sa respecte sabloanele din folderul 'sabloane'.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>4. Apasati butonul corespunzator pentru a importa datele.</t>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>3. Configurati Compatibilitati si ReguliRotunjire daca e necesar.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>5. Selectati fisierul .xlsx si asteptati confirmarea importului.</t>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>4. Apasati GENERARE NECESAR pentru a calcula necesarul.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>5. Rezultatul apare in sheet-ul Necesar.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="19">
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B10:B11"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B5:C5"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="C14:C15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -748,12 +804,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Cod Produs</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Stoc Depozit</t>
         </is>
@@ -780,12 +836,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Cod Produs</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Cantitate Vanzare</t>
         </is>
@@ -804,33 +860,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>Cod Produs</t>
-        </is>
-      </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Cod Produs Original</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Cod Produs Compatibil</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
-        <is>
-          <t>Observatii</t>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>EXEMPLU_COD_VECHI</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>EXEMPLU_COD_NOU</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>COD_DISCONTINUAT</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>COD_INLOCUITOR</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C1"/>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -842,94 +916,168 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>Categorie / Cod Produs</t>
-        </is>
-      </c>
-      <c r="B1" s="12" t="inlineStr">
-        <is>
-          <t>Unitate Masura</t>
-        </is>
-      </c>
-      <c r="C1" s="12" t="inlineStr">
-        <is>
-          <t>Rotunjire La</t>
-        </is>
-      </c>
-      <c r="D1" s="12" t="inlineStr">
-        <is>
-          <t>Tip Rotunjire</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>buc</t>
-        </is>
-      </c>
-      <c r="C2" s="13" t="n">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Categorie</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>Descriere</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>Sus (Ceiling)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>EXEMPLU_COD_1</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="C3" s="14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D3" s="14" t="inlineStr">
-        <is>
-          <t>Sus (Ceiling)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>EXEMPLU_COD_2</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>buc</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Sus (Ceiling)</t>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>Rotunjire la multiplu de 10. Valori sub 5 devin 10. Exemplu: 3-&gt;10, 12-&gt;10, 15-&gt;20, 27-&gt;30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>Rotunjire la numar par (multiplu de 2). Exemplu: 1-&gt;2, 3-&gt;4, 5-&gt;6, 7-&gt;8</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Rotunjire la multiplu de 5. Valori 1-2 devin 0 (se elimina). Exemplu: 2-&gt;0, 3-&gt;5, 7-&gt;5, 8-&gt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Rotunjire la multiplu de 5 cu minim 5 daca stoc depozit &lt; 3. Exemplu: 2-&gt;5(daca stoc&lt;3), 8-&gt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Cod</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Denumire</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Categorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>2700000075968</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Folie de laminare 200 microni 10/18 cm</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>2700000089538</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Folie de laminare 130 microni 10/18 cm</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>2700000286197</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Folie Silicon Urban Protekt Clear Pro</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="006A1B9A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Cod Produs</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>Vanzare</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>Necesar</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>Observatii</t>
         </is>
       </c>
     </row>
@@ -939,7 +1087,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00757575"/>
@@ -956,22 +1104,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Data/Ora</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Operatiune</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Detalii</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>

</xml_diff>

<commit_message>
perf: Rewrite VBA to use in-memory arrays and bulk operations
Performance optimizations:
- All sheet reads use Range.Value -> Variant array (bulk read)
- All sheet writes use Range.Resize.Value = array (bulk write)
- No more cell-by-cell iteration for formatting (range-based)
- Dictionary loading via generic LoadDictFromSheet with array read
- Source files closed immediately after array read
- Application.EnableEvents = False during operations
- Erase arrays after use to free memory
- Log writes use 1x4 array instead of 4 cell writes

Functional changes:
- Necesar sheet now includes Stoc Depozit column (5 cols total):
  Cod Produs | Vanzare | Stoc Depozit | Necesar | Observatii

https://claude.ai/code/session_01WLPgVpN32fAC7hpn167gUT
</commit_message>
<xml_diff>
--- a/NecesarAprovizionare.xlsx
+++ b/NecesarAprovizionare.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'StocDepozit'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'VanzariMagazin'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Compatibilitati'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Necesar'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Necesar'!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1050,13 +1050,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1072,17 +1073,22 @@
       </c>
       <c r="C1" s="13" t="inlineStr">
         <is>
+          <t>Stoc Depozit</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
           <t>Necesar</t>
         </is>
       </c>
-      <c r="D1" s="13" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Observatii</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: Rename StocDepozit->StocMagazin, 4-col Compatibilitati, Text format, borders
Changes:
- Rename StocDepozit to StocMagazin everywhere (sheets, VBA, templates, README)
- Compatibilitati now 4 columns: Cod Original | Denumire Original |
  Cod Compatibil | Denumire Compatibil (VBA reads col A->C for mapping)
- Column A (Cod Produs) set to Text format BEFORE data write to preserve
  leading zeros on product codes
- Borders applied on all data ranges (import, necesar, log entries)
- ApplyBorders helper for consistent thin borders across sheets

https://claude.ai/code/session_01WLPgVpN32fAC7hpn167gUT
</commit_message>
<xml_diff>
--- a/NecesarAprovizionare.xlsx
+++ b/NecesarAprovizionare.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Meniu" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="StocDepozit" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="StocMagazin" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="VanzariMagazin" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Compatibilitati" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="ReguliRotunjire" sheetId="5" state="visible" r:id="rId5"/>
@@ -16,9 +16,9 @@
     <sheet name="Log" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'StocDepozit'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'StocMagazin'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'VanzariMagazin'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Compatibilitati'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Compatibilitati'!$A$1:$D$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Necesar'!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,11 +89,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00999999"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -167,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -198,19 +193,15 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -610,12 +601,12 @@
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>IMPORT STOC DEPOZIT</t>
+          <t>IMPORT STOC MAGAZIN</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Importa stocul din depozit. Format: CodProdus | Stoc</t>
+          <t>Importa stocul magazinului. Format: CodProdus | Stoc</t>
         </is>
       </c>
     </row>
@@ -676,7 +667,7 @@
     <row r="20">
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Stoc Depozit:</t>
+          <t>Stoc Magazin:</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -811,7 +802,7 @@
       </c>
       <c r="B1" s="13" t="inlineStr">
         <is>
-          <t>Stoc Depozit</t>
+          <t>Stoc Magazin</t>
         </is>
       </c>
     </row>
@@ -860,11 +851,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -875,36 +868,22 @@
       </c>
       <c r="B1" s="13" t="inlineStr">
         <is>
+          <t>Denumire Produs Original</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
           <t>Cod Produs Compatibil</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>EXEMPLU_COD_VECHI</t>
-        </is>
-      </c>
-      <c r="B2" s="14" t="inlineStr">
-        <is>
-          <t>EXEMPLU_COD_NOU</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>COD_DISCONTINUAT</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>COD_INLOCUITOR</t>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>Denumire Produs Compatibil</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B1"/>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -916,7 +895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -925,54 +904,54 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Categorie</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>Descriere</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="16" t="n">
+      <c r="A2" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>Rotunjire la multiplu de 10. Valori sub 5 devin 10. Exemplu: 3-&gt;10, 12-&gt;10, 15-&gt;20, 27-&gt;30</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="16" t="n">
+      <c r="A3" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>Rotunjire la numar par (multiplu de 2). Exemplu: 1-&gt;2, 3-&gt;4, 5-&gt;6, 7-&gt;8</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="16" t="n">
+      <c r="A4" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>Rotunjire la multiplu de 5. Valori 1-2 devin 0 (se elimina). Exemplu: 2-&gt;0, 3-&gt;5, 7-&gt;5, 8-&gt;10</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>Rotunjire la multiplu de 5 cu minim 5 daca stoc depozit &lt; 3. Exemplu: 2-&gt;5(daca stoc&lt;3), 8-&gt;10</t>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Rotunjire la multiplu de 5 cu minim 5 daca stoc magazin &lt; 3. Exemplu: 2-&gt;5(daca stoc&lt;3), 8-&gt;10</t>
         </is>
       </c>
     </row>
@@ -991,51 +970,6 @@
         <is>
           <t>Categorie</t>
         </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>2700000075968</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Folie de laminare 200 microni 10/18 cm</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>2700000089538</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Folie de laminare 130 microni 10/18 cm</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>2700000286197</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Folie Silicon Urban Protekt Clear Pro</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1073,7 +1007,7 @@
       </c>
       <c r="C1" s="13" t="inlineStr">
         <is>
-          <t>Stoc Depozit</t>
+          <t>Stoc Magazin</t>
         </is>
       </c>
       <c r="D1" s="13" t="inlineStr">

</xml_diff>

<commit_message>
feat: Smart necesar formula with daily average and configurable days
New formula: Necesar = MAX(0, CEILING((Vanzare/ZileVanz) * ZileNec - Stoc))
- Configurable settings on Meniu sheet (C33=Zile vanzare, C34=Zile necesar)
- Validates settings before generation (both must be > 0)
- Calculates daily average, projects for target days, subtracts stock
- Rounds up to integer, then applies category rounding if applicable
- Necesar sheet now 6 columns: Cod | Vanzare | Medie/Zi | Stoc | Necesar | Obs
- Status shows calculation parameters (e.g. "30z vanz / 7z nec")

https://claude.ai/code/session_01WLPgVpN32fAC7hpn167gUT
</commit_message>
<xml_diff>
--- a/NecesarAprovizionare.xlsx
+++ b/NecesarAprovizionare.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'StocMagazin'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'VanzariMagazin'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Compatibilitati'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Necesar'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Necesar'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,6 +87,18 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="002F5496"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
@@ -100,7 +112,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -129,6 +141,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C62828"/>
         <bgColor rgb="00C62828"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+        <bgColor rgb="00FFF3E0"/>
       </patternFill>
     </fill>
     <fill>
@@ -162,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -191,15 +209,19 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -568,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C31"/>
+  <dimension ref="B2:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -743,19 +765,53 @@
     <row r="30">
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>4. Apasati GENERARE NECESAR pentru a calcula necesarul.</t>
+          <t>4. Setati zilele de vanzare si necesar mai jos.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>5. Rezultatul apare in sheet-ul Necesar.</t>
+          <t>5. Apasati GENERARE NECESAR pentru a calcula necesarul.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>SETARI CALCUL</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Zile vanzare:</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Zile necesar:</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>Formula: Necesar = CEILING((Vanzare / ZileVanz) * ZileNec) - Stoc</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="21">
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="B3:C3"/>
@@ -773,6 +829,8 @@
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B7:B8"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="C18:C19"/>
     <mergeCell ref="C14:C15"/>
   </mergeCells>
@@ -795,12 +853,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Cod Produs</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Stoc Magazin</t>
         </is>
@@ -827,12 +885,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Cod Produs</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Cantitate Vanzare</t>
         </is>
@@ -861,22 +919,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Cod Produs Original</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Denumire Produs Original</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Cod Produs Compatibil</t>
         </is>
       </c>
-      <c r="D1" s="13" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>Denumire Produs Compatibil</t>
         </is>
@@ -904,69 +962,69 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Categorie</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Descriere</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="15" t="n">
+      <c r="A2" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Rotunjire la multiplu de 10. Valori sub 5 devin 10. Exemplu: 3-&gt;10, 12-&gt;10, 15-&gt;20, 27-&gt;30</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="15" t="n">
+      <c r="A3" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>Rotunjire la numar par (multiplu de 2). Exemplu: 1-&gt;2, 3-&gt;4, 5-&gt;6, 7-&gt;8</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="15" t="n">
+      <c r="A4" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Rotunjire la multiplu de 5. Valori 1-2 devin 0 (se elimina). Exemplu: 2-&gt;0, 3-&gt;5, 7-&gt;5, 8-&gt;10</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="15" t="n">
+      <c r="A5" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Rotunjire la multiplu de 5 cu minim 5 daca stoc magazin &lt; 3. Exemplu: 2-&gt;5(daca stoc&lt;3), 8-&gt;10</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Cod</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Denumire</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Categorie</t>
         </is>
@@ -984,45 +1042,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Cod Produs</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Vanzare</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>Medie/Zi</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>Stoc Magazin</t>
         </is>
       </c>
-      <c r="D1" s="13" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>Necesar</t>
         </is>
       </c>
-      <c r="E1" s="13" t="inlineStr">
+      <c r="F1" s="15" t="inlineStr">
         <is>
           <t>Observatii</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1"/>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1044,22 +1108,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Data/Ora</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Operatiune</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Detalii</t>
         </is>
       </c>
-      <c r="D1" s="13" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>Status</t>
         </is>

</xml_diff>